<commit_message>
Toma C14 sin interruptor: fuera el interruptor rojo que se veía en el lateral
- CAD: la toma C14 con interruptor (B08Z6FCR5Z) pasa a una con
  portafusibles y sin interruptor (B07CQ54BY4). Recorte del cajón, taladros
  M3 a 36 mm, ventana de la carcasa 38 × 46 y topes; 0 choques y recorridos
  sin roces.
- Lista de compra (#15, total 636,02 €), MONTAJE GENERAL (W2 y W3 directos
  a la fuente, sin W4/W5; protocolo del apartado 4.1; figura 1), PASO A
  PASO (P1.1, P4.1, P4.3, P4.4), pendientes, índice, aviso en la ficha #15
  y fichas que cableaban el interruptor.
- DECISIONES: la máquina se apaga desenchufándola; el fusible en un solo
  polo sigue abierto.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MDyCaz223X6sxbbMPeRyMY
</commit_message>
<xml_diff>
--- a/carcasa/diseno-A/Lista_de_piezas.xlsx
+++ b/carcasa/diseno-A/Lista_de_piezas.xlsx
@@ -237,7 +237,7 @@
     <t xml:space="preserve">STEP_piezas/A-C04.step</t>
   </si>
   <si>
-    <t xml:space="preserve">Ventana de acceso a la toma C14 (38 × 56), rejillas, ranura 2.1 × 90 de la tapa interior con muesca R8 encima; ranura 4×14 de la leva; agujero Ø6,5 de la antena</t>
+    <t xml:space="preserve">Ventana del enchufe de la toma C14 (38 × 46), rejillas, ranura 2.1 × 90 de la tapa interior con muesca R8 encima; ranura 4×14 de la leva; agujero Ø6,5 de la antena</t>
   </si>
   <si>
     <t xml:space="preserve">A-C05</t>
@@ -648,7 +648,7 @@
     <t xml:space="preserve">STEP_piezas/A-K05.step</t>
   </si>
   <si>
-    <t xml:space="preserve">Recorte de la toma C14 (47,9 × 28,2) y 2 taladros M3</t>
+    <t xml:space="preserve">Recorte de la toma C14 (31.90 × 27.65, ancho × alto) y 2 taladros M3 a 36 mm, uno encima de otro</t>
   </si>
   <si>
     <t xml:space="preserve">A-K06</t>
@@ -942,13 +942,13 @@
     <t xml:space="preserve">E07</t>
   </si>
   <si>
-    <t xml:space="preserve">Toma C14 con fusible e interruptor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B08Z6FCR5Z</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.amazon.es/dp/B08Z6FCR5Z</t>
+    <t xml:space="preserve">Toma C14 con portafusibles, sin interruptor (Cablepelado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B07CQ54BY4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.amazon.es/dp/B07CQ54BY4</t>
   </si>
   <si>
     <t xml:space="preserve">E07.1</t>
@@ -2142,15 +2142,15 @@
       </c>
       <c r="H5" s="6" t="n">
         <f aca="false">'A Fabricar'!I51/1000</f>
-        <v>7.795</v>
+        <v>7.805</v>
       </c>
       <c r="I5" s="7" t="n">
         <f aca="false">'A Comprar'!I53</f>
-        <v>882.1</v>
+        <v>882.43</v>
       </c>
       <c r="J5" s="7" t="n">
         <f aca="false">'A Comprar'!I54</f>
-        <v>866.12</v>
+        <v>866.45</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>17</v>
@@ -2479,7 +2479,7 @@
         <v>1.5</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="J10" s="4" t="s">
         <v>69</v>
@@ -3543,7 +3543,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
         <v>204</v>
       </c>
@@ -3569,7 +3569,7 @@
         <v>1.5</v>
       </c>
       <c r="I39" s="9" t="n">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="J39" s="4" t="s">
         <v>206</v>
@@ -4015,7 +4015,7 @@
       <c r="H51" s="11"/>
       <c r="I51" s="12" t="n">
         <f aca="false">SUM(I5:I50)</f>
-        <v>7795</v>
+        <v>7805</v>
       </c>
       <c r="J51" s="11"/>
       <c r="K51" s="11"/>
@@ -4288,7 +4288,7 @@
       </c>
       <c r="K10" s="4"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
         <v>305</v>
       </c>
@@ -4309,11 +4309,11 @@
         <v>1</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>7.7</v>
+        <v>8.03</v>
       </c>
       <c r="I11" s="7" t="n">
         <f aca="false">G11*H11</f>
-        <v>7.7</v>
+        <v>8.03</v>
       </c>
       <c r="J11" s="4" t="s">
         <v>309</v>
@@ -5749,7 +5749,7 @@
       <c r="H53" s="11"/>
       <c r="I53" s="16" t="n">
         <f aca="false">SUM(I5:I52)</f>
-        <v>882.1</v>
+        <v>882.43</v>
       </c>
       <c r="J53" s="11"/>
       <c r="K53" s="11"/>
@@ -5760,7 +5760,7 @@
       </c>
       <c r="I54" s="17" t="n">
         <f aca="false">I53-SUMIF(A5:A52,"M09",I5:I52)</f>
-        <v>866.12</v>
+        <v>866.45</v>
       </c>
     </row>
   </sheetData>
@@ -5771,7 +5771,7 @@
     <hyperlink ref="D8" r:id="rId4" display="https://www.amazon.es/dp/B0BNJPL4MW"/>
     <hyperlink ref="D9" r:id="rId5" display="https://www.amazon.es/dp/B0CBW6THN1"/>
     <hyperlink ref="D10" r:id="rId6" display="https://www.amazon.es/dp/B06XWRCWZ9"/>
-    <hyperlink ref="D11" r:id="rId7" display="https://www.amazon.es/dp/B08Z6FCR5Z"/>
+    <hyperlink ref="D11" r:id="rId7" display="https://www.amazon.es/dp/B07CQ54BY4"/>
     <hyperlink ref="D12" r:id="rId8" display="https://www.amazon.es/dp/B09XB58ZXJ"/>
     <hyperlink ref="D13" r:id="rId9" display="https://www.amazon.es/dp/B07V86XPL4"/>
     <hyperlink ref="D14" r:id="rId10" display="https://www.amazon.es/dp/B07Q495GQG"/>

</xml_diff>

<commit_message>
Carcasa a 100 mm de fondo (antes 103)
- Hueco detrás del cajón de componentes de 14 a 11 mm; el cajón y su interior no cambian.
- Espárrago de tierra de la carcasa cortado a 8 mm (con 10 quedaba a 1 mm del cajón).
- Puente de tierra W10 recolocado; asidero derecho referido a la trasera del cajón.
- Regenerados STEP, DXF, visor 3D, conexiones y lista de piezas.
- 0 choques, barridos limpios, mismos avisos de cables que con 103 mm.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MDyCaz223X6sxbbMPeRyMY
</commit_message>
<xml_diff>
--- a/carcasa/diseno-A/Lista_de_piezas.xlsx
+++ b/carcasa/diseno-A/Lista_de_piezas.xlsx
@@ -620,7 +620,7 @@
         <v>220</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>442.5</v>
@@ -1042,13 +1042,13 @@
         <v>439.5</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H9" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>362</v>
+        <v>352</v>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
@@ -1096,13 +1096,13 @@
         <v>439.5</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H10" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>489</v>
+        <v>474</v>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Ventana del enchufe de la toma C14 (38 × 46), rejillas, ranura 2.1 × 90 de la tapa interior con muesca R8 encima; ranura 4×14 de la leva; agujero Ø6,5 de la antena</t>
+          <t>Ventana del enchufe de la toma C14 (38 × 46), rejillas, ranura 2.1 × 87 de la tapa interior con muesca R8 encima; ranura 4×14 de la leva; agujero Ø6,5 de la antena</t>
         </is>
       </c>
     </row>
@@ -1150,13 +1150,13 @@
         <v>220</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
@@ -1200,13 +1200,13 @@
         <v>217</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H12" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I12" s="9" t="n">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
@@ -1254,13 +1254,13 @@
         <v>218</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>10.5</v>
+        <v>7.5</v>
       </c>
       <c r="H13" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I13" s="9" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
@@ -1308,13 +1308,13 @@
         <v>218</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>10.5</v>
+        <v>7.5</v>
       </c>
       <c r="H14" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
@@ -1362,13 +1362,13 @@
         <v>218.3</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>89.59999999999999</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="H15" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I15" s="9" t="n">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
@@ -1470,13 +1470,13 @@
         <v>217</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>12.5</v>
+        <v>9.5</v>
       </c>
       <c r="H17" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I17" s="9" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Soldado a la trasera; 12.5 mm de vuelo. Hace de guía de la tapa interior</t>
+          <t>Soldado a la trasera; 9.5 mm de vuelo. Hace de guía de la tapa interior</t>
         </is>
       </c>
     </row>
@@ -1632,13 +1632,13 @@
         <v>222</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="H20" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I20" s="9" t="n">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="F22" s="6" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G22" s="6" t="n">
         <v>37.5</v>
@@ -1746,7 +1746,7 @@
         <v>1.5</v>
       </c>
       <c r="I22" s="9" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
@@ -1848,13 +1848,13 @@
         <v>216</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="H24" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I24" s="9" t="n">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
@@ -2002,13 +2002,13 @@
         <v>145.2</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H27" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I27" s="9" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
@@ -2052,13 +2052,13 @@
         <v>147.7</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="H28" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I28" s="9" t="n">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
@@ -2106,13 +2106,13 @@
         <v>145.2</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H29" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I29" s="9" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
@@ -2156,13 +2156,13 @@
         <v>145.2</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H30" s="6" t="n">
         <v>1.5</v>
       </c>
       <c r="I30" s="9" t="n">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>

</xml_diff>